<commit_message>
Team addresses as IAR named them; Outreach is part of Da'wah
The launch teams' group addresses are now a fixed list (TEAM_SLUGS in
teams.ts) instead of being worked out from each name: portal-team-tech@
(IT Services), -maintenance@, -security@, -welfare@, -hw@, -cafe@,
-imams@, -seniors@, -page@, -sports@ and so on. Queue roles, team email,
IT & Maintenance, go-live, the members template, the demo and the docs
use them. Outreach is dropped (26 teams); rows for it in an older copy of
the members Sheet count for Da'wah.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpLQsK7BmjTGF9a3ho3RHS
</commit_message>
<xml_diff>
--- a/ops/go-live/members-template.xlsx
+++ b/ops/go-live/members-template.xlsx
@@ -305,7 +305,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-facility-maintenance@islam1.org</t>
+          <t xml:space="preserve">portal-team-maintenance@islam1.org</t>
         </is>
       </c>
     </row>
@@ -329,7 +329,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-health-wellness@islam1.org</t>
+          <t xml:space="preserve">portal-team-hw@islam1.org</t>
         </is>
       </c>
     </row>
@@ -341,7 +341,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-iar-cafe@islam1.org</t>
+          <t xml:space="preserve">portal-team-cafe@islam1.org</t>
         </is>
       </c>
     </row>
@@ -353,7 +353,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-imam-office@islam1.org</t>
+          <t xml:space="preserve">portal-team-imams@islam1.org</t>
         </is>
       </c>
     </row>
@@ -365,7 +365,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-it-services@islam1.org</t>
+          <t xml:space="preserve">portal-team-tech@islam1.org</t>
         </is>
       </c>
     </row>
@@ -389,127 +389,137 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-older-adult-community@islam1.org</t>
+          <t xml:space="preserve">portal-team-seniors@islam1.org</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outreach</t>
+          <t xml:space="preserve">Page Road</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-outreach@islam1.org</t>
+          <t xml:space="preserve">portal-team-page@islam1.org</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page Road</t>
+          <t xml:space="preserve">Safety &amp; Security</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-page-road@islam1.org</t>
+          <t xml:space="preserve">portal-team-security@islam1.org</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Safety &amp; Security</t>
+          <t xml:space="preserve">Shura</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-safety-security@islam1.org</t>
+          <t xml:space="preserve">portal-team-shura@islam1.org</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shura</t>
+          <t xml:space="preserve">Social &amp; Welfare</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-shura@islam1.org</t>
+          <t xml:space="preserve">portal-team-welfare@islam1.org</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social &amp; Welfare</t>
+          <t xml:space="preserve">Sports &amp; Recreation</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-social-welfare@islam1.org</t>
+          <t xml:space="preserve">portal-team-sports@islam1.org</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sports &amp; Recreation</t>
+          <t xml:space="preserve">Volunteer</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-sports-recreation@islam1.org</t>
+          <t xml:space="preserve">portal-team-volunteer@islam1.org</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Volunteer</t>
+          <t xml:space="preserve">Women's Committee</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-volunteer@islam1.org</t>
+          <t xml:space="preserve">portal-team-women@islam1.org</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Women's Committee</t>
+          <t xml:space="preserve">Youth</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-women@islam1.org</t>
+          <t xml:space="preserve">portal-team-youth@islam1.org</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Youth</t>
+          <t xml:space="preserve">Portal: IAR office</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-team-youth@islam1.org</t>
+          <t xml:space="preserve">portal-role-office@islam1.org</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Member</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The IAR office: rentals, run sheet; can submit for any committee</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portal: IAR office</t>
+          <t xml:space="preserve">Portal: Finance</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-role-office@islam1.org</t>
+          <t xml:space="preserve">portal-role-finance@islam1.org</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -519,19 +529,19 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">The IAR office: rentals, run sheet; can submit for any committee</t>
+          <t xml:space="preserve">Finance review, payment, QuickBooks entry, restricted S&amp;W requests</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portal: Finance</t>
+          <t xml:space="preserve">Portal: Executive</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-role-finance@islam1.org</t>
+          <t xml:space="preserve">portal-role-executive@islam1.org</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -541,19 +551,19 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finance review, payment, QuickBooks entry, restricted S&amp;W requests</t>
+          <t xml:space="preserve">Whoever holds an executive office (Head Imam, Shura chair, CEO): final mission review of events, executive approvals</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portal: Executive</t>
+          <t xml:space="preserve">Portal: Admins</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">portal-role-executive@islam1.org</t>
+          <t xml:space="preserve">portal-role-admin@islam1.org</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -562,28 +572,6 @@
         </is>
       </c>
       <c r="E31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Whoever holds an executive office (Head Imam, Shura chair, CEO): final mission review of events, executive approvals</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Portal: Admins</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">portal-role-admin@islam1.org</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Member</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
         <is>
           <t xml:space="preserve">Two or three people who support the portal. Never approve or pay</t>
         </is>
@@ -844,91 +832,84 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outreach</t>
+          <t xml:space="preserve">Page Road</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page Rd</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page Road</t>
+          <t xml:space="preserve">Safety &amp; Security</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page Rd</t>
+          <t xml:space="preserve">Safety and Security Expenses</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Safety &amp; Security</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Safety and Security Expenses</t>
+          <t xml:space="preserve">Shura</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shura</t>
+          <t xml:space="preserve">Social &amp; Welfare</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Social &amp; Welfare</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social &amp; Welfare</t>
+          <t xml:space="preserve">Sports &amp; Recreation</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social &amp; Welfare</t>
+          <t xml:space="preserve">Sports &amp; Recreation Expenses</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sports &amp; Recreation</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sports &amp; Recreation Expenses</t>
+          <t xml:space="preserve">Volunteer</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Volunteer</t>
+          <t xml:space="preserve">Women's Committee</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Women Expenses</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Women's Committee</t>
+          <t xml:space="preserve">Youth</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Women Expenses</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Youth</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
         <is>
           <t xml:space="preserve">Youth Expenses</t>
         </is>

</xml_diff>